<commit_message>
update npm dependencies (#19)
</commit_message>
<xml_diff>
--- a/public/zcl_excel_demo1.xlsx
+++ b/public/zcl_excel_demo1.xlsx
@@ -124,8 +124,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="1" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -413,10 +413,10 @@
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>44561</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>0.2488078703703704</v>
       </c>
     </row>

</xml_diff>